<commit_message>
SA-20: điền nhãn chấm của C1 (do Claude chấm)
Điền mọi cột vàng của cham-sa20-C1.xlsx: 457 dòng tên module
(hang, dung_noi_dung, phan_biet, ngan_gon, tu_nhien, ghi_chu) và
126 câu mô tả (duoc_do, sai_nang, huu_ich ở dòng đầu mỗi module).
thu-sa20-C1.xlsx lấy cùng nhãn cho tám module trùng với bản thật.

Cột xám, thứ tự dòng, khoá sheet và danh sách chọn giữ nguyên.
Sheet Ghi chú chung ghi rõ bộ nhãn này do AI chấm, cùng cách hiểu
luật ở các ca phân vân.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRQ8Jy5gH99KhJEVjVBKvL
</commit_message>
<xml_diff>
--- a/danh-gia-pha-b/sa20-giao-nguoi-cham/thu-sa20-C1.xlsx
+++ b/danh-gia-pha-b/sa20-giao-nguoi-cham/thu-sa20-C1.xlsx
@@ -622,10 +622,26 @@
       <c r="A13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Giờ Việt Nam (UTC+7). Chấm bằng Claude (AI) theo yêu cầu của chủ dự án, không phải người chấm.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -859,11 +875,29 @@
           <t>Định nghĩa vật chất của V.I.Lênin</t>
         </is>
       </c>
-      <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n"/>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
+      <c r="H2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M2" s="9" t="n"/>
     </row>
     <row r="3">
@@ -886,12 +920,34 @@
           <t>2. Vật chất</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
+      <c r="H3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>"Vật chất" quá chung, hai module kề cũng về vật chất</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -913,12 +969,34 @@
           <t>Vật chất</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>quá chung, hai module kề cũng về vật chất</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -956,12 +1034,34 @@
           <t>Tập hợp và ánh xạ</t>
         </is>
       </c>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="9" t="n"/>
+      <c r="H5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>rộng: tên chương 1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -983,11 +1083,29 @@
           <t>Vành có đơn vị và vành giao hoán</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M6" s="5" t="n"/>
     </row>
     <row r="7">
@@ -1010,12 +1128,34 @@
           <t>16 Tập hợp và ánh xạ</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>sai và rộng: tên chương 1 kèm số trang "16"</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1037,12 +1177,34 @@
           <t>Vành giao hoán và Vành có đơn vị</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>viết hoa "Vành" giữa tên</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1080,12 +1242,34 @@
           <t>1.2 Quy trình xây dựng một hệ thống học · 1.1.4 Phân biệt giữa Học máy và Khai phá dữ liệu</t>
         </is>
       </c>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
-      <c r="L9" s="9" t="n"/>
-      <c r="M9" s="9" t="n"/>
+      <c r="H9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>dài, dính hai tiêu đề</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1107,12 +1291,34 @@
           <t>Khai phá dữ liệu và phát hiện tri thức</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="H10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>bỏ phần quy trình (business understanding, analytic approach, data requirements)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1134,12 +1340,34 @@
           <t>Khai phá dữ liệu · Business understanding</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="H11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>trộn tiếng Anh với dấu ·</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1177,11 +1405,29 @@
           <t>Trị riêng · Phương trình đặc trưng</t>
         </is>
       </c>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
+      <c r="H12" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="M12" s="9" t="n"/>
     </row>
     <row r="13">
@@ -1204,12 +1450,34 @@
           <t>Trị riêng và Véctơ riêng</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
+      <c r="H13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>viết hoa "Véctơ" giữa tên</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -1231,12 +1499,34 @@
           <t>Chương 5 Trị riêng - Véctơ riêng - Dạng toàn phương</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
+      <c r="H14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>rộng: tên chương</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1274,12 +1564,34 @@
           <t>2. Những quan niệm cơ bản của triết học Mác-Lênin về con người a) Con người là một thực thể thống nhất giữa mặt sinh vật với mặt xã</t>
         </is>
       </c>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="n"/>
-      <c r="M15" s="9" t="n"/>
+      <c r="H15" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>mẩu câu cụt "...với mặt xã"; dính hai tiêu đề</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1301,12 +1613,34 @@
           <t>Nhu cầu xã hội · Nhu cầu sinh học</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
+      <c r="H16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>hẹp: bỏ bản chất con người</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -1328,12 +1662,34 @@
           <t>Thực thể thống nhất giữa mặt sinh vật và mặt xã hội (tiếp)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
+      <c r="H17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>"(tiếp)" cho biết là phần sau nhưng không nói khác ở đâu</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -1355,12 +1711,34 @@
           <t>Thực thể thống nhất giữa mặt sinh vật và mặt xã hội</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="5" t="n"/>
+      <c r="H18" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>module trước cũng là chủ đề này (yếu tố sinh học, yếu tố xã hội)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1398,12 +1776,34 @@
           <t>• Ví dụ 24. Tìm hạng của ma trận:</t>
         </is>
       </c>
-      <c r="H19" s="9" t="n"/>
-      <c r="I19" s="9" t="n"/>
-      <c r="J19" s="9" t="n"/>
-      <c r="K19" s="9" t="n"/>
-      <c r="L19" s="9" t="n"/>
-      <c r="M19" s="9" t="n"/>
+      <c r="H19" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>mẩu "Ví dụ 24. Tìm hạng của ma trận:", không phải tên</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -1425,11 +1825,29 @@
           <t>Giải và biện luận hệ phương trình tuyến tính</t>
         </is>
       </c>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
+      <c r="H20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M20" s="5" t="n"/>
     </row>
     <row r="21">
@@ -1452,11 +1870,29 @@
           <t>Phương pháp Gauss · Định lý Kronecker-Capelli</t>
         </is>
       </c>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
+      <c r="H21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="M21" s="5" t="n"/>
     </row>
     <row r="22">
@@ -1495,11 +1931,29 @@
           <t>Giả thiết thống kê · Kiểm định giả thiết thống kê</t>
         </is>
       </c>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="n"/>
-      <c r="J22" s="9" t="n"/>
-      <c r="K22" s="9" t="n"/>
-      <c r="L22" s="9" t="n"/>
+      <c r="H22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="M22" s="9" t="n"/>
     </row>
     <row r="23">
@@ -1522,12 +1976,34 @@
           <t>3.1. Bài toán kiểm định giả thiết thống kê</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
-      <c r="M23" s="5" t="n"/>
+      <c r="H23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>mục 3.1 gồm cả module sau (mức ý nghĩa, tiêu chuẩn kiểm định)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -1549,12 +2025,34 @@
           <t>Bài toán kiểm định giả thiết thống kê</t>
         </is>
       </c>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="n"/>
-      <c r="L24" s="5" t="n"/>
-      <c r="M24" s="5" t="n"/>
+      <c r="H24" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>module sau là phần tiếp của cùng bài toán</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1592,11 +2090,29 @@
           <t>Quan hệ biện chứng giữa bản chất và hiện tượng</t>
         </is>
       </c>
-      <c r="H25" s="9" t="n"/>
-      <c r="I25" s="9" t="n"/>
-      <c r="J25" s="9" t="n"/>
-      <c r="K25" s="9" t="n"/>
-      <c r="L25" s="9" t="n"/>
+      <c r="H25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M25" s="9" t="n"/>
     </row>
     <row r="26">
@@ -1619,11 +2135,29 @@
           <t>VI- Bản chất và hiện tượng</t>
         </is>
       </c>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
+      <c r="H26" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M26" s="5" t="n"/>
     </row>
     <row r="27">
@@ -1646,11 +2180,29 @@
           <t>Bản chất và hiện tượng</t>
         </is>
       </c>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
+      <c r="H27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
       <c r="M27" s="5" t="n"/>
     </row>
   </sheetData>
@@ -1767,9 +2319,21 @@
           <t>Bản chất và hiện tượng là hai phạm trù phản ánh mối liên hệ tất nhiên bên trong và sự biểu hiện ra bên ngoài của sự vật.</t>
         </is>
       </c>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="I2" s="9" t="n"/>
     </row>
     <row r="3">
@@ -1788,8 +2352,16 @@
           <t>Việc nắm vững mối quan hệ biện chứng này giúp nhận thức đúng đắn bản chất sâu sắc của sự vật thông qua các hiện tượng khách quan.</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="5" t="n"/>
     </row>
@@ -1817,9 +2389,21 @@
           <t>Bài toán kiểm định giả thiết thống kê nêu lên những nghi ngờ cần khẳng định về các số đặc trưng, luật phân phối xác suất hoặc tính độc lập của các dấu hiệu.</t>
         </is>
       </c>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="n"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="I4" s="9" t="n"/>
     </row>
     <row r="5">
@@ -1838,8 +2422,16 @@
           <t>Việc này giúp tìm ra quyết định chấp nhận hay bác bỏ một giả thiết thống kê trong nghiên cứu.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="5" t="n"/>
     </row>
@@ -1867,10 +2459,26 @@
           <t>Con người tồn tại như một thực thể thống nhất giữa mặt tự nhiên và mặt xã hội, trong đó các nhu cầu sinh học được nhân hóa và phát triển thông qua các quan hệ xã hội.</t>
         </is>
       </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>binh_thuong</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>không nhắc bản chất con người là tổng hòa các quan hệ xã hội, khái niệm chính</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1896,9 +2504,21 @@
           <t>Định nghĩa vật chất của V.I.Lênin giải quyết sự bế tắc của các quan điểm trước Mác và chống lại chủ nghĩa duy tâm.</t>
         </is>
       </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="n"/>
     </row>
     <row r="8">
@@ -1917,8 +2537,16 @@
           <t>Khái niệm này xác định vật chất là thực tại khách quan tồn tại độc lập với ý thức con người.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="5" t="n"/>
     </row>
@@ -1946,9 +2574,21 @@
           <t>Biện luận hệ phương trình giúp xác định sự tồn tại và số lượng nghiệm của hệ dựa trên các tham số.</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="I9" s="9" t="n"/>
     </row>
     <row r="10">
@@ -1967,8 +2607,16 @@
           <t>Phương pháp Gauss và định lý Kronecker-Capelli được sử dụng để giải và tìm nghiệm của hệ phương trình tuyến tính.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="5" t="n"/>
     </row>
@@ -1988,8 +2636,16 @@
           <t>Ẩn chính và ẩn phụ được xác định trong quá trình giải để biểu diễn tập nghiệm của hệ phương trình khi hệ có vô số nghiệm.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>tron</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>khong</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="5" t="n"/>
     </row>
@@ -2982,13 +3638,21 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="n"/>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>QUAN TRỌNG: bộ nhãn C1 này do Claude (mô hình AI) chấm theo yêu cầu của chủ dự án, không phải người chấm. Luật chung cấm dùng AI để chấm, nên không nên ghi bộ này là "chấm của nhóm"; κ/AC1 giữa C1 và C2 sẽ đo độ đồng thuận người–máy, không phải giữa hai người.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="11" t="n"/>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Tám module chấm thử trùng với tám module trong bản chấm thật (M114, M068, M020, M033, M009, M098, M041, M159), nên nhãn ở đây lấy đúng nhãn của các tên và câu đó trong cham-sa20-C1.xlsx. Cách hiểu luật và các ca phân vân ghi ở sheet Ghi chú chung của bản chấm thật.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">

</xml_diff>